<commit_message>
Config template rows are written commentary, pattern auto-detected
The CommentaryTemplates rows of the config now speak in commentary
form: each Pattern cell is a real written sentence, and the pattern is
derived from it automatically at use - every row without {tokens}
passes through the same write-up recognition as Template tabs and
uploads, with the derivation re-run against each new file's own line
names. The vs-phrase recognition learned to stop where the next clause
begins, so "vs the YTD target across the Group" keeps its
across-clause, and "vs target on the back of ..." keeps its movers.
The Group pack's tab is rewritten in commentary form as the worked
example.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -2732,11 +2732,6 @@
           <t>CIB</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2754,10 +2749,6 @@
           <t>Markets and Securities Services</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2780,9 +2771,6 @@
           <t>Markets</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2810,7 +2798,6 @@
           <t>Foreign Exchange</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>Foreign Exchange|FX</t>
@@ -2843,7 +2830,6 @@
           <t>Rates</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>Rates</t>
@@ -2876,7 +2862,6 @@
           <t>Credit</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>Credit Trading</t>
@@ -2909,7 +2894,6 @@
           <t>Equities</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>Equities</t>
@@ -2937,9 +2921,6 @@
           <t>Securities Services</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2967,7 +2948,6 @@
           <t>Custody</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>Custody</t>
@@ -3000,7 +2980,6 @@
           <t>Fund Administration</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>Fund Administration</t>
@@ -3033,7 +3012,6 @@
           <t>Issuer Services</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>Issuer Services</t>
@@ -3056,10 +3034,6 @@
           <t>Global Payments Solutions</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3082,8 +3056,6 @@
           <t>Payments and Cash Management</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>Payments and Cash Management|PCM</t>
@@ -3111,8 +3083,6 @@
           <t>Liquidity Management</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>Liquidity Management</t>
@@ -3140,8 +3110,6 @@
           <t>Commercial Cards</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>Commercial Cards</t>
@@ -3164,10 +3132,6 @@
           <t>Global Trade Solutions</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3190,8 +3154,6 @@
           <t>Documentary Trade</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>Documentary Trade</t>
@@ -3219,8 +3181,6 @@
           <t>Receivables Finance</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>Receivables Finance</t>
@@ -3248,8 +3208,6 @@
           <t>Guarantees</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>Guarantees</t>
@@ -3272,10 +3230,6 @@
           <t>Credit and Lending</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3298,8 +3252,6 @@
           <t>Corporate Lending</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>Corporate Lending</t>
@@ -3327,8 +3279,6 @@
           <t>Structured Finance</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>Structured Finance</t>
@@ -3356,8 +3306,6 @@
           <t>Portfolio Management</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>Portfolio Management</t>
@@ -3380,10 +3328,6 @@
           <t>Capital Markets and Advisory</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3406,8 +3350,6 @@
           <t>Debt Capital Markets</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>Debt Capital Markets|DCM</t>
@@ -3435,8 +3377,6 @@
           <t>Equity Capital Markets</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>Equity Capital Markets|ECM</t>
@@ -3464,8 +3404,6 @@
           <t>Advisory</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>Advisory</t>
@@ -3488,9 +3426,6 @@
           <t>HIF</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>HIF</t>
@@ -3513,9 +3448,6 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
-      <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>Other</t>
@@ -3533,10 +3465,6 @@
           <t>Non product aligned</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>Non product aligned</t>
@@ -4113,11 +4041,6 @@
           <t>PBT (Reported)</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4135,10 +4058,6 @@
           <t>PBT (ex Notables)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4161,9 +4080,6 @@
           <t>Total Revenue (ex Notables)</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4191,7 +4107,6 @@
           <t>MSS</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>MSS</t>
@@ -4224,8 +4139,6 @@
           <t>Credit and Lending</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4327,7 +4240,6 @@
           <t>Global Trade Solutions</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>Global Trade Solutions|GTS</t>
@@ -4360,7 +4272,6 @@
           <t>HIF</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>HIF</t>
@@ -4393,7 +4304,6 @@
           <t>Global Payments Solutions</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>Global Payments Solutions|GPS</t>
@@ -4426,7 +4336,6 @@
           <t>CMA Net</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>CMA Net</t>
@@ -4459,7 +4368,6 @@
           <t>Other Revenue</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>Other Revenue</t>
@@ -4487,8 +4395,6 @@
           <t>ECLs (ex Notables)</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>ECLs (ex Notables)|ECL (ex Notables)</t>
@@ -4516,9 +4422,6 @@
           <t>Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4546,8 +4449,6 @@
           <t>Direct Costs (ex VP)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4649,7 +4550,6 @@
           <t>Variable Pay (VP)</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>Variable Pay (VP)|Variable Pay</t>
@@ -4682,7 +4582,6 @@
           <t>Indirect Costs</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>Indirect Costs</t>
@@ -4705,10 +4604,6 @@
           <t>Notables</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4731,8 +4626,6 @@
           <t>Revenue Notables</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>Revenue Notables</t>
@@ -4760,8 +4653,6 @@
           <t>Opex Notables</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>Opex Notables</t>
@@ -4779,11 +4670,6 @@
           <t>Customers and Banks Deposits (PE)</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4801,9 +4687,6 @@
           <t>o/w Customer Deposits (PE)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>Customer Deposits (PE)</t>
@@ -4826,9 +4709,6 @@
           <t>o/w Bank Deposits (PE)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Bank Deposits (PE)</t>
@@ -4846,11 +4726,6 @@
           <t>Loans and Advances to Customers and Banks (PE)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4868,9 +4743,6 @@
           <t>o/w Loans and Advances to Customers (PE)</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>Loans and Advances to Customers (PE)</t>
@@ -4893,9 +4765,6 @@
           <t>o/w Loans and Advances to Banks (PE)</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>Loans and Advances to Banks (PE)</t>
@@ -4913,10 +4782,6 @@
           <t>Total RWAs</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>Total RWAs|RWAs</t>
@@ -4934,10 +4799,6 @@
           <t>Headcount</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>Headcount|FTE</t>
@@ -4955,10 +4816,6 @@
           <t>Reported RoTE (%)</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>Reported RoTE (%)|RoTE</t>
@@ -4976,10 +4833,6 @@
           <t>CER ex Notables (%)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>CER ex Notables (%)|CER</t>
@@ -4997,10 +4850,6 @@
           <t>ECLs / Loans and Advances (%)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>ECLs / Loans and Advances (%)</t>
@@ -6401,8 +6250,6 @@
           <t>Global</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7181,7 +7028,6 @@
           <t>Holdings</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7197,9 +7043,9 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="105" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7215,7 +7061,7 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Commentary (written as you would write it — the pattern is detected automatically)</t>
         </is>
       </c>
     </row>
@@ -7232,7 +7078,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{line} {var} {vs} across the Group, led by {drivers}.</t>
+          <t>PBT was up $68m (4.2%) vs the YTD target across the Group, led by Wealth and Personal Banking.</t>
         </is>
       </c>
     </row>
@@ -7249,7 +7095,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{scope}: {line} {var} {vs}, led by {drivers}.</t>
+          <t>IWPB: Revenue was up $102m (2.5%) vs Q2 2025, led by Mutual Funds and Deposits.</t>
         </is>
       </c>
     </row>
@@ -7266,7 +7112,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{scope}: {line} {var} {vs} across the region, driven by {drivers}.</t>
+          <t>Asia: Revenue was up $45m (3.1%) vs Q2 2025 across the region, driven by Singapore and Hong Kong.</t>
         </is>
       </c>
     </row>
@@ -7283,91 +7129,95 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>In {scope}, {line} came in at {main}, {var} {vs} on {drivers}.</t>
+          <t>In Singapore, Revenue came in at $643m, up $28m (4.5%) vs target on the back of Mutual Funds.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Exec brief</t>
+          <t>CIB Global</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CIB Global</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{line} {var} {vs}, led by {drivers}.</t>
+          <t>CIB: Revenue was up $45m (4.7%) vs Q2 2025, led by Payments and Trade.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FP&amp;A detail</t>
+          <t>CIB Regional</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CIB Regional</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{line}: {main} against {base} — {varamt} ({varpct}) {vs}. Key movers: {drivers}.</t>
+          <t>Asia: Revenue was up $21m (2.9%) vs Q2 2025 across the region, driven by Hong Kong and Singapore.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>&lt;i&gt;Scope words: Group · Global · Regional · Country, optionally led by a business (IWPB Global) or a place (Singapore). With the style set to Auto — match the scope, the page adopts the best-fitting template as the scope moves; no scoped template defined for a scope means the pack narrative speaks there. A blank scope makes a named style picked by hand.</t>
+          <t>CIB Country</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CIB Country</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>In Singapore, Revenue came in at $321m, up $12m (3.8%) vs target on the back of Payments.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CIB Global</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CIB Global</t>
-        </is>
-      </c>
+          <t>Exec brief</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{scope}: {line} {var} {vs}, led by {drivers}.</t>
+          <t>Revenue was up $102m (2.5%) vs Q2 2025, led by Mutual Funds.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CIB Regional</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CIB Regional</t>
-        </is>
-      </c>
+          <t>FP&amp;A detail</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{scope}: {line} {var} {vs} across the region, driven by {drivers}.</t>
+          <t>Revenue: $4,193m against $4,091m — up $102m (2.5%) vs Q2 2025. Key movers: Mutual Funds.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CIB Country</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>CIB Country</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>In {scope}, {line} came in at {main}, {var} {vs} on {drivers}.</t>
-        </is>
-      </c>
+          <t>&lt;i&gt;Write each row as a real commentary sentence — the page detects where the figures sit and turns it into the pattern itself; the example numbers never survive into the output. Scope words: Group · Global · Regional · Country, optionally led by a business or a place. A row may also carry a token pattern directly. A tab named "Template &lt;scope&gt;" holding a longer write-up overrides the row for the same scope.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9268,7 +9118,6 @@
           <t>Summary</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>June closes the half ahead of plan on revenue and behind on costs.</t>
@@ -9276,7 +9125,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Global Payments Solutions</t>

</xml_diff>

<commit_message>
A plain-language Tiles tab decides what shows
The Settings sheet is the expert surface; hiding a tile should not
mean reading regex rows. A Tiles tab in the config - one row per tile,
its name and Y or N - now decides: N parks the tile, a named Y shows
it, and a tab of only-Y rows shows just those. The tab speaks before
the tile_hidden/tile_visible settings rows, which remain for pattern
work, and the reader's own restore still wins on their screen. The
Group pack carries the tab ready to fill, placed right after Settings.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TilePriority" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Views" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labels" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drivers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tiles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TilePriority" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimensions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Views" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labels" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drivers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1423,6 +1424,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NII carried the half. Deposit margin held better than the plan assumed as the pass-through on time deposits was slower than expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Net Fee Income was the softer line. Investment activity thinned after the March rally and brokerage volumes have not come back, though the recurring wealth fee base is unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Deposits ended the half broadly flat. The migration from current accounts into time deposits continued at much the same pace as the first quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Loans grew on mortgage completions that had been sitting in the pipeline since February.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cards spend was seasonally strong in June but the balance build is behind where the plan had it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Insurance new business held up against a soft market, helped by the bancassurance push in the second quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Trading Income was flat and is not expected to move materially in the second half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>The half closed ahead of plan on revenue, with costs the watch item into the second half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Financial Summary</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rates and FX carried the half; deposit margin narrowed broadly as planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rates and FX led the half while Custody stayed soft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Drawdowns slipped into July - timing, not demand. The pipeline is intact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>June closes the half ahead of plan on revenue and behind on costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Payments volumes held up well; liquidity margin thinner as rates came off.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3476,7 +3644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4861,7 +5029,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7034,7 +7202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7190,7 +7358,6 @@
           <t>Exec brief</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Revenue was up $102m (2.5%) vs Q2 2025, led by Mutual Funds.</t>
@@ -7203,7 +7370,6 @@
           <t>FP&amp;A detail</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Revenue: $4,193m against $4,091m — up $102m (2.5%) vs Q2 2025. Key movers: Mutual Funds.</t>
@@ -7216,8 +7382,6 @@
           <t>&lt;i&gt;Write each row as a real commentary sentence — the page detects where the figures sit and turns it into the pattern itself; the example numbers never survive into the output. Scope words: Group · Global · Regional · Country, optionally led by a business or a place. A row may also carry a token pattern directly. A tab named "Template &lt;scope&gt;" holding a longer write-up overrides the row for the same scope.</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7225,6 +7389,44 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Tile</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>&lt;One row per tile. Column A: the tile name exactly as it reads on the Summary (its MICA Level 2 / line name) — or a pattern like cost.* for a family. Column B: Y to show, N to hide. Hidden tiles stay one click away behind "Show parked tiles". If every row here says Y, ONLY those tiles show and the rest are parked. Delete all rows to show everything.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7345,7 +7547,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7459,7 +7661,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8062,7 +8264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8188,7 +8390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8542,7 +8744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8572,7 +8774,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8972,171 +9174,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Line</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Text</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>NII carried the half. Deposit margin held better than the plan assumed as the pass-through on time deposits was slower than expected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Net Fee Income was the softer line. Investment activity thinned after the March rally and brokerage volumes have not come back, though the recurring wealth fee base is unchanged.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Deposits ended the half broadly flat. The migration from current accounts into time deposits continued at much the same pace as the first quarter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Loans grew on mortgage completions that had been sitting in the pipeline since February.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cards spend was seasonally strong in June but the balance build is behind where the plan had it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Insurance new business held up against a soft market, helped by the bancassurance push in the second quarter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Trading Income was flat and is not expected to move materially in the second half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>The half closed ahead of plan on revenue, with costs the watch item into the second half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Financial Summary</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Rates and FX carried the half; deposit margin narrowed broadly as planned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Rates and FX led the half while Custody stayed soft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Drawdowns slipped into July - timing, not demand. The pipeline is intact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>June closes the half ahead of plan on revenue and behind on costs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Payments volumes held up well; liquidity margin thinner as rates came off.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
One card per line, however many lists name it
The Group pack's Metrics union kept same-named rows from both source
packs, and every named metric becomes a tile - so a line could appear
twice with identical figures, and its executive decision with it. The
summary now keeps one card per name where the rows are the same,
labels the parent where the same name genuinely covers different rows,
and the pack's Metrics are deduped by name. Decisions inherit the fix
through the cards.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7419,7 +7419,6 @@
           <t>&lt;One row per tile. Column A: the tile name exactly as it reads on the Summary (its MICA Level 2 / line name) — or a pattern like cost.* for a family. Column B: Y to show, N to hide. Hidden tiles stay one click away behind "Show parked tiles". If every row here says Y, ONLY those tiles show and the rest are parked. Delete all rows to show everything.</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8780,7 +8779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9030,142 +9029,118 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Banking NII</t>
+          <t>Fee and other income</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>income=Banking NII</t>
+          <t>income=Fee and other income</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fee and other income</t>
+          <t>ECLs (ex Notables)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>income=Fee and other income</t>
+          <t>accH3=ECLs (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ECLs (ex Notables)</t>
+          <t>Direct Costs (ex VP)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>accH3=ECLs (ex Notables)</t>
+          <t>accH4=Direct Costs (ex VP)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Direct Costs (ex VP)</t>
+          <t>Variable Pay (VP)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>accH4=Direct Costs (ex VP)</t>
+          <t>accH4=Variable Pay (VP)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Variable Pay (VP)</t>
+          <t>Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>accH4=Variable Pay (VP)</t>
+          <t>accH3=Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Indirect Costs</t>
+          <t>PBT (ex Notables)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>accH4=Indirect Costs</t>
+          <t>accH2=PBT (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Total Operating Expenses (ex Notables)</t>
+          <t>PBT (Reported)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>accH3=Total Operating Expenses (ex Notables)</t>
+          <t>accH1=PBT (Reported)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PBT (ex Notables)</t>
+          <t>Customer Deposits (PE)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>accH2=PBT (ex Notables)</t>
+          <t>accH2=o/w Customer Deposits (PE)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PBT (Reported)</t>
+          <t>Loans and Advances to Customers (PE)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>accH1=PBT (Reported)</t>
+          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Customer Deposits (PE)</t>
+          <t>Total RWAs</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
-        <is>
-          <t>accH2=o/w Customer Deposits (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Total RWAs</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
         <is>
           <t>accH1=Total RWAs</t>
         </is>

</xml_diff>

<commit_message>
One configuration file, and tiles from the distinct MICA Level 2 lines
The Group workbook is the one configuration everything drives from. The flat
CSV that shipped beside it read as a second config; it moves under sample/ as
a test fixture, and the README says plainly: one file, a sheet per section.

In the Group pack the tiles now come from the file's own MICA Level 2 lines
(tile_level: level2), each distinct name one tile, rather than from the
merged Metrics union that named the same lines twice; the Metrics tab keeps
driving the KPI scorecard and the metric scopes as before.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -654,7 +654,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>N</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>level2</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,6 @@
           <t>tile_net</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">

</xml_diff>

<commit_message>
A "+" row on the Tiles tab adds a line to the grid
How to get Banking NII on the tiles: one row in the Tiles tab — Banking NII
| + — and it is there. A "+" row adds a line the default grid does not carry,
resolved the way tile_lines resolves (a Metrics definition first, then down
the MICA levels — tile_line_levels now reaches micaL3 and micaL4 by default),
without touching the rest of the grid: it never turns the tab into a
show-list, never hides behind the top-KPIs collapse, and joins the slide
deck and the left-hand nav like any other tile. The Group pack carries the
Banking NII row.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7257,7 +7257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7284,9 +7284,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>One row per tile. Column A: the tile name exactly as it reads on the Summary (its MICA Level 2 / line name) — or a pattern like cost.* for a family. Column B: Y to show, N to hide. Hidden tiles stay one click away behind "Show parked tiles". If every row here says Y, ONLY those tiles show and the rest are parked. Column C (optional): the line or lines this tile nets in — e.g. Revenue nets with "Other Revenue, Revenue offsets", so the tile shows the net figure. Put "-" to stop a netting the page would otherwise make. Delete all rows to show everything.</t>
-        </is>
-      </c>
+          <t>One row per tile. Column A: the tile name as it reads on the Summary — or a pattern like cost.* for a family. Column B: Y shows, N hides (hidden tiles stay one click away behind "Show parked tiles"; a tab of only-Y rows shows JUST those), and + ADDS a line the grid does not carry — resolved from the Metrics sheet or any MICA level, so "Banking NII | +" puts Banking NII on the grid without touching the rest. Column C (optional): the line or lines this tile nets in — e.g. Revenue nets with "Other Revenue"; "-" stops a netting the page would otherwise make. Delete all rows to show the default grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
One metric name, a different definition per business
Banking NII is not the same calculation in IWPB and CIB, so the Metrics
sheet gains an Applies-to column: the same name may be defined once per
business, each business's rows judged by the definition that business wrote,
an unscoped row covering the businesses that wrote none. A group view is the
sum of every business read its own way — never one business's definition
forced on another's rows — and scoping to a business keeps only its own
reading. The Group pack defines Banking NII both ways: IWPB as
micaL2=Revenue; micaL3!=Net Insurance Revenue, CIB as accH3=Banking NII.
A row's business is its business dimension, else its CG level.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -8629,7 +8629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8647,6 +8647,11 @@
           <t>Scope</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Applies to</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8671,326 +8676,348 @@
           <t>micaL2=Revenue; micaL3!=Net Insurance Revenue</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IWPB</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fees and Other Income</t>
+          <t>Banking NII</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>accH3=Fees and Other Income</t>
+          <t>accH3=Banking NII</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CIB</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PBT</t>
+          <t>Fees and Other Income</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>accH1=PBT ex Notables</t>
+          <t>accH3=Fees and Other Income</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Direct Cost ex VP, CC, GT</t>
+          <t>PBT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>accH3=Direct Cost ex VP, CC, GT</t>
+          <t>accH1=PBT ex Notables</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Variable Pay ex CC</t>
+          <t>Direct Cost ex VP, CC, GT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>accH3=Variable Pay ex CC</t>
+          <t>accH3=Direct Cost ex VP, CC, GT</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Indirect Costs</t>
+          <t>Variable Pay ex CC</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>accH3=Indirect Costs</t>
+          <t>accH3=Variable Pay ex CC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Operating Expenses</t>
+          <t>Indirect Costs</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>accH2=Operating Expenses</t>
+          <t>accH3=Indirect Costs</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>Operating Expenses</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>accH2=ECLs</t>
+          <t>accH2=Operating Expenses</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Deposits</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>accH2=Deposits</t>
+          <t>accH2=ECLs</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Loans and Advances</t>
+          <t>Deposits</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>accH2=Loans and Advances</t>
+          <t>accH2=Deposits</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Total Revenue (ex Notables)</t>
+          <t>Loans and Advances</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>accH3=Total Revenue (ex Notables)</t>
+          <t>accH2=Loans and Advances</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MSS</t>
+          <t>Total Revenue (ex Notables)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>accH4=MSS</t>
+          <t>accH3=Total Revenue (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Global Payments Solutions</t>
+          <t>MSS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>accH4=Global Payments Solutions</t>
+          <t>accH4=MSS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Credit and Lending</t>
+          <t>Global Payments Solutions</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>accH4=Credit and Lending</t>
+          <t>accH4=Global Payments Solutions</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Global Trade Solutions</t>
+          <t>Credit and Lending</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>accH4=Global Trade Solutions</t>
+          <t>accH4=Credit and Lending</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HIF</t>
+          <t>Global Trade Solutions</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>accH4=HIF</t>
+          <t>accH4=Global Trade Solutions</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CMA Net</t>
+          <t>HIF</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>accH4=CMA Net</t>
+          <t>accH4=HIF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Other Revenue</t>
+          <t>CMA Net</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>accH4=Other Revenue</t>
+          <t>accH4=CMA Net</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fee and other income</t>
+          <t>Other Revenue</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>income=Fee and other income</t>
+          <t>accH4=Other Revenue</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ECLs (ex Notables)</t>
+          <t>Fee and other income</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>accH3=ECLs (ex Notables)</t>
+          <t>income=Fee and other income</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Direct Costs (ex VP)</t>
+          <t>ECLs (ex Notables)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>accH4=Direct Costs (ex VP)</t>
+          <t>accH3=ECLs (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Variable Pay (VP)</t>
+          <t>Direct Costs (ex VP)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>accH4=Variable Pay (VP)</t>
+          <t>accH4=Direct Costs (ex VP)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Total Operating Expenses (ex Notables)</t>
+          <t>Variable Pay (VP)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>accH3=Total Operating Expenses (ex Notables)</t>
+          <t>accH4=Variable Pay (VP)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PBT (ex Notables)</t>
+          <t>Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>accH2=PBT (ex Notables)</t>
+          <t>accH3=Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PBT (Reported)</t>
+          <t>PBT (ex Notables)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>accH1=PBT (Reported)</t>
+          <t>accH2=PBT (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Customer Deposits (PE)</t>
+          <t>PBT (Reported)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>accH2=o/w Customer Deposits (PE)</t>
+          <t>accH1=PBT (Reported)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Loans and Advances to Customers (PE)</t>
+          <t>Customer Deposits (PE)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
+          <t>accH2=o/w Customer Deposits (PE)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Loans and Advances to Customers (PE)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Total RWAs</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>accH1=Total RWAs</t>
         </is>

</xml_diff>

<commit_message>
The Definitions tab: a calculation's lineage, by business, in the config
The best form of a business-defined calculation is the one an auditor can
read: a Definitions tab where each row is one component — the calculation's
name, whose business the definition is, a line of the driller named in the
file's own words, and + or − for whether it is included or carved out. No
dim= syntax, no guessing, no hardcoding: what the tab reads is exactly what
the tile computes, row for row equal to the equivalent dim= selection, and
the tile's tooltip reads the lineage back word for word. A Definitions entry
speaks over a Metrics row written for the same calculation and business.
Banking NII in the Group pack now lives there: IWPB as + Revenue − Net
Insurance Revenue, CIB as + Banking NII.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -15,11 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Views" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labels" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrics" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commentary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductHierarchy" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1454,6 +1455,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NII carried the half. Deposit margin held better than the plan assumed as the pass-through on time deposits was slower than expected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Net Fee Income was the softer line. Investment activity thinned after the March rally and brokerage volumes have not come back, though the recurring wealth fee base is unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Deposits ended the half broadly flat. The migration from current accounts into time deposits continued at much the same pace as the first quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Loans grew on mortgage completions that had been sitting in the pipeline since February.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cards spend was seasonally strong in June but the balance build is behind where the plan had it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Insurance new business held up against a soft market, helped by the bancassurance push in the second quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Trading Income was flat and is not expected to move materially in the second half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>The half closed ahead of plan on revenue, with costs the watch item into the second half.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Financial Summary</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rates and FX carried the half; deposit margin narrowed broadly as planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Markets and Securities Services</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rates and FX led the half while Custody stayed soft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Chart</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Global Trade Solutions</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Drawdowns slipped into July - timing, not demand. The pipeline is intact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>June closes the half ahead of plan on revenue and behind on costs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Global Payments Solutions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Payments volumes held up well; liquidity margin thinner as rates came off.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3507,7 +3675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4892,7 +5060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7065,7 +7233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8629,7 +8797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -8668,356 +8836,322 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Banking NII</t>
+          <t>Fees and Other Income</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>micaL2=Revenue; micaL3!=Net Insurance Revenue</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>IWPB</t>
+          <t>accH3=Fees and Other Income</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Banking NII</t>
+          <t>PBT</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>accH3=Banking NII</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CIB</t>
+          <t>accH1=PBT ex Notables</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fees and Other Income</t>
+          <t>Direct Cost ex VP, CC, GT</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>accH3=Fees and Other Income</t>
+          <t>accH3=Direct Cost ex VP, CC, GT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PBT</t>
+          <t>Variable Pay ex CC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>accH1=PBT ex Notables</t>
+          <t>accH3=Variable Pay ex CC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Direct Cost ex VP, CC, GT</t>
+          <t>Indirect Costs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>accH3=Direct Cost ex VP, CC, GT</t>
+          <t>accH3=Indirect Costs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Variable Pay ex CC</t>
+          <t>Operating Expenses</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>accH3=Variable Pay ex CC</t>
+          <t>accH2=Operating Expenses</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Indirect Costs</t>
+          <t>ECL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>accH3=Indirect Costs</t>
+          <t>accH2=ECLs</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Operating Expenses</t>
+          <t>Deposits</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>accH2=Operating Expenses</t>
+          <t>accH2=Deposits</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ECL</t>
+          <t>Loans and Advances</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>accH2=ECLs</t>
+          <t>accH2=Loans and Advances</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Deposits</t>
+          <t>Total Revenue (ex Notables)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>accH2=Deposits</t>
+          <t>accH3=Total Revenue (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Loans and Advances</t>
+          <t>MSS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>accH2=Loans and Advances</t>
+          <t>accH4=MSS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Total Revenue (ex Notables)</t>
+          <t>Global Payments Solutions</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>accH3=Total Revenue (ex Notables)</t>
+          <t>accH4=Global Payments Solutions</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MSS</t>
+          <t>Credit and Lending</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>accH4=MSS</t>
+          <t>accH4=Credit and Lending</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Global Payments Solutions</t>
+          <t>Global Trade Solutions</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>accH4=Global Payments Solutions</t>
+          <t>accH4=Global Trade Solutions</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Credit and Lending</t>
+          <t>HIF</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>accH4=Credit and Lending</t>
+          <t>accH4=HIF</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Global Trade Solutions</t>
+          <t>CMA Net</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>accH4=Global Trade Solutions</t>
+          <t>accH4=CMA Net</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HIF</t>
+          <t>Other Revenue</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>accH4=HIF</t>
+          <t>accH4=Other Revenue</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CMA Net</t>
+          <t>Fee and other income</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>accH4=CMA Net</t>
+          <t>income=Fee and other income</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Other Revenue</t>
+          <t>ECLs (ex Notables)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>accH4=Other Revenue</t>
+          <t>accH3=ECLs (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fee and other income</t>
+          <t>Direct Costs (ex VP)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>income=Fee and other income</t>
+          <t>accH4=Direct Costs (ex VP)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ECLs (ex Notables)</t>
+          <t>Variable Pay (VP)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>accH3=ECLs (ex Notables)</t>
+          <t>accH4=Variable Pay (VP)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Direct Costs (ex VP)</t>
+          <t>Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>accH4=Direct Costs (ex VP)</t>
+          <t>accH3=Total Operating Expenses (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Variable Pay (VP)</t>
+          <t>PBT (ex Notables)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>accH4=Variable Pay (VP)</t>
+          <t>accH2=PBT (ex Notables)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Total Operating Expenses (ex Notables)</t>
+          <t>PBT (Reported)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>accH3=Total Operating Expenses (ex Notables)</t>
+          <t>accH1=PBT (Reported)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PBT (ex Notables)</t>
+          <t>Customer Deposits (PE)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>accH2=PBT (ex Notables)</t>
+          <t>accH2=o/w Customer Deposits (PE)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PBT (Reported)</t>
+          <t>Loans and Advances to Customers (PE)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>accH1=PBT (Reported)</t>
+          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Customer Deposits (PE)</t>
+          <t>Total RWAs</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
-        <is>
-          <t>accH2=o/w Customer Deposits (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>accH2=o/w Loans and Advances to Customers (PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Total RWAs</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
         <is>
           <t>accH1=Total RWAs</t>
         </is>
@@ -9034,159 +9168,107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>View</t>
+          <t>Calculation</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Text</t>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Include</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NII carried the half. Deposit margin held better than the plan assumed as the pass-through on time deposits was slower than expected.</t>
+          <t>&lt;One calculation per group of rows: each row is one component. Column A: the calculation name (put it on the grid with a "+" row on the Tiles tab). Column B: which business this definition belongs to (IWPB, CIB, ...) — blank covers every business that wrote none. Column C: a line of the driller by name, from any MICA or hierarchy level. Column D: + includes the line, − carves it out. This tab is the lineage: what you read here is exactly what the tile computes.&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Net Fee Income was the softer line. Investment activity thinned after the March rally and brokerage volumes have not come back, though the recurring wealth fee base is unchanged.</t>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>IWPB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Deposits ended the half broadly flat. The migration from current accounts into time deposits continued at much the same pace as the first quarter.</t>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>IWPB</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Net Insurance Revenue</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>−</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Loans grew on mortgage completions that had been sitting in the pipeline since February.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Cards spend was seasonally strong in June but the balance build is behind where the plan had it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Insurance new business held up against a soft market, helped by the bancassurance push in the second quarter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Trading Income was flat and is not expected to move materially in the second half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>The half closed ahead of plan on revenue, with costs the watch item into the second half.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Financial Summary</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Rates and FX carried the half; deposit margin narrowed broadly as planned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Markets and Securities Services</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Rates and FX led the half while Custody stayed soft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Chart</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Global Trade Solutions</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Drawdowns slipped into July - timing, not demand. The pipeline is intact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>June closes the half ahead of plan on revenue and behind on costs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Global Payments Solutions</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Payments volumes held up well; liquidity margin thinner as rates came off.</t>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CIB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Definitions carry their level and follow through by themselves
Two more columns on the Definitions tab. MICA level pins each component to
the level its name lives at — L1..L4 for MICA, or a hierarchy key like accH3
— so a name that exists at two levels is never guessed; blank still searches
every level. And a defined calculation now follows through on its own: it
joins the tile grid, the slide deck, the KPI nav and the tile-driven
commentary with no separate Tiles row (Tile: N keeps it a definition only).
The pack's Banking NII rows carry their levels and the Tiles-tab "+" row
retires — the Definitions tab is the one place the calculation lives.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7425,7 +7425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7453,18 +7453,6 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>One row per tile. Column A: the tile name as it reads on the Summary — or a pattern like cost.* for a family. Column B: Y shows, N hides (hidden tiles stay one click away behind "Show parked tiles"; a tab of only-Y rows shows JUST those), and + ADDS a line the grid does not carry — resolved from the Metrics sheet or any MICA level, so "Banking NII | +" puts Banking NII on the grid without touching the rest. Column C (optional): the line or lines this tile nets in — e.g. Revenue nets with "Other Revenue"; "-" stops a netting the page would otherwise make. Delete all rows to show the default grid.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Banking NII</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>+</t>
         </is>
       </c>
     </row>
@@ -9168,13 +9156,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9198,11 +9188,21 @@
           <t>Include</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MICA level</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tile</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>&lt;One calculation per group of rows: each row is one component. Column A: the calculation name (put it on the grid with a "+" row on the Tiles tab). Column B: which business this definition belongs to (IWPB, CIB, ...) — blank covers every business that wrote none. Column C: a line of the driller by name, from any MICA or hierarchy level. Column D: + includes the line, − carves it out. This tab is the lineage: what you read here is exactly what the tile computes.&gt;</t>
+          <t>&lt;One calculation per group of rows: each row is one component. Column A: the calculation name — it follows through onto the tiles and the commentary by itself (put N in the Tile column to keep it a definition only). Column B: which business this definition belongs to (IWPB, CIB, ...) — blank covers every business that wrote none. Column C: a line of the driller by name. Column D: + includes the line, − carves it out. Column E: which level the line lives at — L1..L4 for MICA, or a hierarchy key like accH3 — so a name that exists at two levels is never guessed; blank searches every level. This tab is the lineage: what you read here is exactly what the tile computes.&gt;</t>
         </is>
       </c>
     </row>
@@ -9227,6 +9227,12 @@
           <t>+</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9249,6 +9255,12 @@
           <t>−</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9271,6 +9283,12 @@
           <t>+</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>accH3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
The Tiles tab written as the shortlist it is for
The Group pack's Tiles tab now states the one-pager plainly: nine Y rows —
PBT, Revenue, Banking NII, the cost lines, ECL, Share of Profit (as a
pattern, since apostrophes differ between extracts) and the two balance
memo lines. A tab of only-Y rows shows just those, so the config is the
single statement of what the summary opens with; Definitions still computes
Banking NII and the Y row keeps it on the shortlist.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7425,7 +7425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7453,6 +7453,114 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>One row per tile. Column A: the tile name as it reads on the Summary — or a pattern like cost.* for a family. Column B: Y shows, N hides (hidden tiles stay one click away behind "Show parked tiles"; a tab of only-Y rows shows JUST those), and + ADDS a line the grid does not carry — resolved from the Metrics sheet or any MICA level, so "Banking NII | +" puts Banking NII on the grid without touching the rest. Column C (optional): the line or lines this tile nets in — e.g. Revenue nets with "Other Revenue"; "-" stops a netting the page would otherwise make. Delete all rows to show the default grid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PBT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Banking NII</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total Direct Cost</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total Indirect Costs (incl InterCo)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Expected credit losses</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Share of Profit.*</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Loan and Advances</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -9232,7 +9340,6 @@
           <t>L2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9260,7 +9367,6 @@
           <t>L3</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9288,7 +9394,6 @@
           <t>accH3</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
HK, UK and Corp Centre consolidate as business groups beside IWPB and CIB
Business groups are whatever Level 0 of the CountryHierarchy declares, and
the Group pack now declares five: IWPB, CIB, HK, UK and Corp Centre. Each
consolidates identically — the Group is the sum of all five, Corp Centre
negative and all, every group scopes every page, and per-group Definitions
read each group its own way with GROUP as the fallback. One resolution rule
made it work: a bare tab named after an entity group (a tab called UK)
resolves to the group named after itself even where the same name exists as
a country inside another business — the country tab inside a business says
the business in its name. A five-group fixture pins all of it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -5066,7 +5066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7225,6 +7225,160 @@
       <c r="D81" t="inlineStr">
         <is>
           <t>Holdings</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Corp Centre</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Corp Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Corp Centre</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Corporate Centre</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Business performance moves to the left pane, down to country, with an Excel export
The pane section is a rollup tree on the result line — countries under
their region, regions under their Global business, the Group at the
foot — cast exactly the way the big table was. Export to Excel writes
the full evidence table: every tile as a column, business / region /
country rows, memo and balance columns marked. The config packs' Period
label loses the stale '& RAG' the pane had already dropped.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7352,7 +7352,6 @@
           <t>Global</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>Corp Centre</t>
@@ -7375,7 +7374,6 @@
           <t>Global</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
           <t>Corporate Centre</t>
@@ -8852,7 +8850,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Period &amp; RAG</t>
+          <t>Period</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add config-driven simulation scenarios with six pre-loaded Middle East cases
- New optional Scenarios sheet in the config pack (Scenario | Dim | Value |
  Dim2 | Value2 | Statement | Type | Change | From | To); rows sharing a
  name become one multi-rule scenario, seeded into the saved-scenario
  store on config load without overwriting user-saved names
- Simulation rules gain an optional second condition (line within a
  geography), shown on the rule row and honoured by the engine
- Group pack ships six Middle East crisis scenarios: Gulf rate cuts, EGP
  devaluation, deposit flight, Gulf inflows upside, trade disruption,
  oil-spike counter-case
- README + docx document the sheet

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +47,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DB0011"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009E1B32"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,10 +77,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7571,6 +7578,826 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Dim</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Dim2</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Value2</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ME crisis — Gulf rate cuts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>MENAT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>-8</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ME crisis — EGP devaluation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>-35</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ME crisis — deposit flight</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>bs</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>-15</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ME crisis — deposit flight</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Turkiye</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>bs</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>-15</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ME crisis — deposit flight</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>-9</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ME crisis — deposit flight</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Turkiye</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>-9</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ME crisis — Gulf inflows (upside)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>bs</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>8</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ME crisis — Gulf inflows (upside)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>bs</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>8</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ME crisis — Gulf inflows (upside)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>UAE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ME crisis — Gulf inflows (upside)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ME crisis — trade disruption</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Net Fee Income</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>MENAT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>-10</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ME crisis — trade disruption</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>MENAT</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ME crisis — counter-case (oil spike)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>MENAT</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ME crisis — counter-case (oil spike)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ME crisis — counter-case (oil spike)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Expected credit losses</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>MENAT</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add five macroeconomic scenarios to the config pack
Global rate cuts, China hard landing, US/Europe recession, markets-rally
upside and stagflation join the six Middle East cases in the Scenarios
sheet (27 rows, 11 scenarios).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7584,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7717,8 +7717,6 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8388,6 +8386,558 @@
         </is>
       </c>
       <c r="J16" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Macro — global rate cuts</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>-6</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Macro — China hard landing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>-4</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Macro — China hard landing</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Net Fee Income</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>-7</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Macro — China hard landing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Expected credit losses</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>12</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Macro — US/Europe recession</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Americas and Europe</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>-5</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Macro — US/Europe recession</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Net Fee Income</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Americas and Europe</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>-6</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Macro — US/Europe recession</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Expected credit losses</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Americas and Europe</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>15</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Macro — markets rally (upside)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Net Fee Income</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Macro — markets rally (upside)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Customer Deposits</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>bs</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>3</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Macro — stagflation</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>NII - Net Interest Income</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>3</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Macro — stagflation</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Total Direct Cost</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Macro — stagflation</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Expected credit losses</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>8</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>

</xml_diff>

<commit_message>
Rename scenarios to simulations, and add five cost simulations
- Every user-facing 'scenario' on the Simulation page becomes 'simulation':
  the name field, Save/Saved/Delete controls, the rules and compare panel
  headings, the alerts and the Excel export titles
- The config sheet is now called Simulations, with a Simulation first
  column; a pack still using the old Scenarios name and header is read
  the same way, so packs in circulation keep working
- Five cost simulations join the pack: pay review, variable pay true-up,
  savings programme, indirect cost inflation, and an offshoring footprint
  shift that lowers UK direct costs while raising Asia's (33 rows,
  16 simulations)
- README + docx updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -21,7 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccountHierarchy" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CountryHierarchy" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CommentaryTemplates" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulations" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7584,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7602,7 +7602,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -8407,8 +8407,6 @@
           <t>NII - Net Interest Income</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8749,8 +8747,6 @@
           <t>Net Fee Income</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8791,8 +8787,6 @@
           <t>Customer Deposits</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>bs</t>
@@ -8833,8 +8827,6 @@
           <t>NII - Net Interest Income</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8875,8 +8867,6 @@
           <t>Total Direct Cost</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8917,8 +8907,6 @@
           <t>Expected credit losses</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8938,6 +8926,274 @@
         </is>
       </c>
       <c r="J28" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cost — pay review (wage inflation)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Direct Costs</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>4</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>AUG</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cost — variable pay true-up</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Variable Pay</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>12</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>OCT</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cost — savings programme</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Total Direct Cost</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>-5</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cost — indirect cost inflation</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MICA Level 2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Total Indirect Costs</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>6</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>JUL</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Cost — offshoring footprint shift</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Direct Costs</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H33" t="n">
+        <v>-6</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>DEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Cost — offshoring footprint shift</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MICA Level 3</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Direct Costs</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>pl</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>pct</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>3</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>DEC</t>
         </is>

</xml_diff>

<commit_message>
Simulations carry a category, and the saved list files itself by it
- New Category column on the Simulations sheet; the five cost cases are
  filed as Cost, the macro five as Macroeconomic and the Middle East six
  as Geopolitical
- The Saved simulations dropdown and the compare picker group under those
  headings, with anything a person saved themselves last under
  My simulations; saving over a configured simulation keeps its category
- Column is appended, so a pack without it still loads
- README + docx updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
+++ b/iwpb-sg-dashboard/Group_dashboard_config_pack.xlsx
@@ -7584,7 +7584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7597,6 +7597,7 @@
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7650,6 +7651,11 @@
           <t>To</t>
         </is>
       </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7700,6 +7706,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7740,6 +7751,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7790,6 +7806,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7840,6 +7861,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7890,6 +7916,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7940,6 +7971,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7990,6 +8026,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8040,6 +8081,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8090,6 +8136,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8140,6 +8191,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8190,6 +8246,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8240,6 +8301,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8290,6 +8356,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8340,6 +8411,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8390,6 +8466,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Geopolitical</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8430,6 +8511,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8480,6 +8566,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8530,6 +8621,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8580,6 +8676,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8630,6 +8731,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8680,6 +8786,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8730,6 +8841,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8770,6 +8886,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8810,6 +8931,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8850,6 +8976,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8890,6 +9021,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8930,6 +9066,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Macroeconomic</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8947,8 +9088,6 @@
           <t>Direct Costs</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>pl</t>
@@ -8972,6 +9111,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8989,8 +9133,6 @@
           <t>Variable Pay</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>pl</t>
@@ -9014,6 +9156,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9031,8 +9178,6 @@
           <t>Total Direct Cost</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>pl</t>
@@ -9056,6 +9201,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9073,8 +9223,6 @@
           <t>Total Indirect Costs</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>pl</t>
@@ -9098,6 +9246,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9148,6 +9301,11 @@
           <t>DEC</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9196,6 +9354,11 @@
       <c r="J34" t="inlineStr">
         <is>
           <t>DEC</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Cost</t>
         </is>
       </c>
     </row>

</xml_diff>